<commit_message>
Rebuild all books with transcript-mining v2 and OTC communications intent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dpaFdbqUZj62BWE6zHYXu
</commit_message>
<xml_diff>
--- a/OTC_BOOK.xlsx
+++ b/OTC_BOOK.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Going Dark" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="NOL Shells" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Foreign OTC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Methodology" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="OTC Intent" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Methodology" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -638,6 +639,21 @@
       <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Cheap foreign lines on currency-neutral ratios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>OTC Intent</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>244</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Management communications signalling buybacks / tenders / capital return.</t>
         </is>
       </c>
     </row>
@@ -656,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -668,6 +684,7 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -691,6 +708,7 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
@@ -739,6 +757,11 @@
           <t>$vol/day k</t>
         </is>
       </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mgmt intent</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -776,6 +799,11 @@
       <c r="I5" s="12" t="n">
         <v>7.6</v>
       </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>△ buyback</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -815,6 +843,11 @@
       <c r="I6" s="13" t="n">
         <v>1</v>
       </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -852,6 +885,11 @@
       <c r="I7" s="12" t="n">
         <v>1.4</v>
       </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -889,6 +927,11 @@
       <c r="I8" s="13" t="n">
         <v>1</v>
       </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -926,6 +969,11 @@
       <c r="I9" s="12" t="n">
         <v>14.6</v>
       </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -963,6 +1011,11 @@
       <c r="I10" s="13" t="n">
         <v>2.8</v>
       </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1000,6 +1053,11 @@
       <c r="I11" s="12" t="n">
         <v>2.8</v>
       </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1037,6 +1095,11 @@
       <c r="I12" s="13" t="n">
         <v>1.6</v>
       </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1074,6 +1137,11 @@
       <c r="I13" s="12" t="n">
         <v>2.1</v>
       </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1113,6 +1181,11 @@
       <c r="I14" s="13" t="n">
         <v>4.3</v>
       </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1150,6 +1223,11 @@
       <c r="I15" s="12" t="n">
         <v>11</v>
       </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1187,6 +1265,11 @@
       <c r="I16" s="13" t="n">
         <v>14.2</v>
       </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1224,6 +1307,11 @@
       <c r="I17" s="12" t="n">
         <v>4.6</v>
       </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -1263,6 +1351,11 @@
       <c r="I18" s="13" t="n">
         <v>6.9</v>
       </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1302,6 +1395,11 @@
       <c r="I19" s="12" t="n">
         <v>16</v>
       </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -1339,6 +1437,11 @@
       <c r="I20" s="13" t="n">
         <v>11.6</v>
       </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>buyback</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="14" t="inlineStr">
@@ -1349,9 +1452,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1363,7 +1466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1375,6 +1478,7 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1398,6 +1502,7 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
@@ -1446,6 +1551,11 @@
           <t>52w pos</t>
         </is>
       </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mgmt intent</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -1481,6 +1591,11 @@
       <c r="I5" s="6" t="n">
         <v>33</v>
       </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1516,6 +1631,11 @@
       <c r="I6" s="9" t="n">
         <v>28</v>
       </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -1551,6 +1671,11 @@
       <c r="I7" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1586,6 +1711,11 @@
       <c r="I8" s="9" t="n">
         <v>3</v>
       </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1621,6 +1751,11 @@
       <c r="I9" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -1656,6 +1791,11 @@
       <c r="I10" s="9" t="n">
         <v>93</v>
       </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1691,6 +1831,11 @@
       <c r="I11" s="6" t="n">
         <v>83</v>
       </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1726,6 +1871,11 @@
       <c r="I12" s="9" t="n">
         <v>20</v>
       </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>▲ tender 4%</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1761,6 +1911,11 @@
       <c r="I13" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1796,6 +1951,11 @@
       <c r="I14" s="9" t="n">
         <v>77</v>
       </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1831,6 +1991,11 @@
       <c r="I15" s="6" t="n">
         <v>53</v>
       </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1866,6 +2031,11 @@
       <c r="I16" s="9" t="n">
         <v>33</v>
       </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>▲ governance</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1901,6 +2071,11 @@
       <c r="I17" s="6" t="n">
         <v>44</v>
       </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -1938,6 +2113,11 @@
       <c r="I18" s="9" t="n">
         <v>36</v>
       </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1973,6 +2153,11 @@
       <c r="I19" s="6" t="n">
         <v>40</v>
       </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -2008,6 +2193,11 @@
       <c r="I20" s="9" t="n">
         <v>41</v>
       </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -2043,6 +2233,11 @@
       <c r="I21" s="6" t="n">
         <v>73</v>
       </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>△ buyback</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -2078,6 +2273,11 @@
       <c r="I22" s="9" t="n">
         <v>98</v>
       </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -2113,6 +2313,11 @@
       <c r="I23" s="6" t="n">
         <v>56</v>
       </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -2148,6 +2353,11 @@
       <c r="I24" s="9" t="n">
         <v>81</v>
       </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>buyback</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -2183,6 +2393,11 @@
       <c r="I25" s="6" t="n">
         <v>57</v>
       </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>▲ buyback 3%</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -2218,6 +2433,11 @@
       <c r="I26" s="9" t="n">
         <v>29</v>
       </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -2253,6 +2473,11 @@
       <c r="I27" s="6" t="n">
         <v>85</v>
       </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -2288,6 +2513,11 @@
       <c r="I28" s="9" t="n">
         <v>44</v>
       </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -2323,6 +2553,11 @@
       <c r="I29" s="6" t="n">
         <v>84</v>
       </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>△ dividend return</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
@@ -2358,6 +2593,11 @@
       <c r="I30" s="9" t="n">
         <v>91</v>
       </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2393,6 +2633,11 @@
       <c r="I31" s="6" t="n">
         <v>96</v>
       </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
@@ -2428,6 +2673,11 @@
       <c r="I32" s="9" t="n">
         <v>23</v>
       </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -2463,6 +2713,11 @@
       <c r="I33" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
@@ -2498,6 +2753,11 @@
       <c r="I34" s="9" t="n">
         <v>1</v>
       </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>strategic review</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2533,6 +2793,11 @@
       <c r="I35" s="6" t="n">
         <v>21</v>
       </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
@@ -2568,6 +2833,11 @@
       <c r="I36" s="9" t="n">
         <v>93</v>
       </c>
+      <c r="J36" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2603,6 +2873,11 @@
       <c r="I37" s="6" t="n">
         <v>38</v>
       </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
@@ -2638,6 +2913,11 @@
       <c r="I38" s="9" t="n">
         <v>97</v>
       </c>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -2673,6 +2953,11 @@
       <c r="I39" s="6" t="n">
         <v>88</v>
       </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
@@ -2708,6 +2993,11 @@
       <c r="I40" s="9" t="n">
         <v>98</v>
       </c>
+      <c r="J40" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2743,6 +3033,11 @@
       <c r="I41" s="6" t="n">
         <v>37</v>
       </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>▲ buyback 2%</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
@@ -2778,6 +3073,11 @@
       <c r="I42" s="9" t="n">
         <v>74</v>
       </c>
+      <c r="J42" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -2813,6 +3113,11 @@
       <c r="I43" s="6" t="n">
         <v>66</v>
       </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
@@ -2848,6 +3153,11 @@
       <c r="I44" s="9" t="n">
         <v>45</v>
       </c>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2883,6 +3193,11 @@
       <c r="I45" s="6" t="n">
         <v>59</v>
       </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
@@ -2918,6 +3233,11 @@
       <c r="I46" s="9" t="n">
         <v>68</v>
       </c>
+      <c r="J46" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -2953,6 +3273,11 @@
       <c r="I47" s="6" t="n">
         <v>66</v>
       </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
@@ -2988,6 +3313,11 @@
       <c r="I48" s="9" t="n">
         <v>31</v>
       </c>
+      <c r="J48" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -3023,6 +3353,11 @@
       <c r="I49" s="6" t="n">
         <v>86</v>
       </c>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
@@ -3058,6 +3393,11 @@
       <c r="I50" s="9" t="n">
         <v>11</v>
       </c>
+      <c r="J50" s="10" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -3093,6 +3433,11 @@
       <c r="I51" s="6" t="n">
         <v>88</v>
       </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="8" t="inlineStr">
@@ -3128,6 +3473,11 @@
       <c r="I52" s="9" t="n">
         <v>71</v>
       </c>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -3165,6 +3515,11 @@
       <c r="I53" s="6" t="n">
         <v>23</v>
       </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
@@ -3200,6 +3555,11 @@
       <c r="I54" s="9" t="n">
         <v>23</v>
       </c>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="14" t="inlineStr">
@@ -3210,9 +3570,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A56:I56"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A56:J56"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3224,7 +3584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3235,6 +3595,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3257,6 +3618,7 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
@@ -3300,6 +3662,11 @@
           <t>Runway yrs</t>
         </is>
       </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Mgmt intent</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -3334,6 +3701,11 @@
       <c r="H5" s="6" t="n">
         <v>1.7</v>
       </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -3370,6 +3742,11 @@
           <t>∞</t>
         </is>
       </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -3406,6 +3783,11 @@
           <t>∞</t>
         </is>
       </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>monetize</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -3440,6 +3822,11 @@
       <c r="H8" s="9" t="n">
         <v>2.7</v>
       </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>strategic review</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -3474,6 +3861,11 @@
       <c r="H9" s="6" t="n">
         <v>1.3</v>
       </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -3508,6 +3900,11 @@
       <c r="H10" s="9" t="n">
         <v>1.1</v>
       </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -3542,6 +3939,11 @@
       <c r="H11" s="6" t="n">
         <v>3.7</v>
       </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -3578,6 +3980,11 @@
           <t>∞</t>
         </is>
       </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -3612,6 +4019,11 @@
       <c r="H13" s="6" t="n">
         <v>18.4</v>
       </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
@@ -3622,9 +4034,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A15:I15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10645,6 +11057,3355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="64" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OTC Intent — management says it will act (calls, press releases, letters)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Most OTC companies never hold a call, so this reads where they do talk: press releases (full text from the wire), SEC 8-K EX-99 exhibits (results, shareholder letters, buyback/tender notices) and calls where they exist — clause-level commitment, negation, new-vs-routine, and the SIZE of any buyback/tender vs market cap. ● = also on a cheapness screen here.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>P/B</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Mcap $M</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Docs 12m</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Evidence (verbatim, dated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>AANNF ●</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Aroundtown S.A.</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>2516.2</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:1</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-26 call] “We continue to execute our share buyback program launched in January, taking advantage of the market volatility and repurchasing our own shares at a significant discount ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>MRETF ●</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Martinrea International</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>520.4</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>call:3 pr:9</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-04 call] “As Pat noted, we sold a majority stake in our fluids plant in China during the quarter, further reducing our presence in the region, and we are exploring other potential ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>HKHGF ●</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Hongkong Land Holdings L</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>18137.9</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>call:1</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-29 call] “Since we launched the buyback, we've invested close to $500,000,000.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>KAEPF ●</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>The Kansai Electric Powe</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>21055.7</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>call:1</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-30 call] “For that, we will generate over JPY 380 billion in cash through asset recycling, including the divestment of our shareholdings.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>TGONF ●</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tetragon Financial Group</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>1136.2</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>call:1 pr:22</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>[2026-04-14 pr] “Tetragon announces the final results of the "modified Dutch auction" tender offer to purchase a portion of the outstanding non-voting shares of Tetragon for a maximum agg”</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>VXRT ●</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Vaxart, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>call:3 ex99:2 letter:3 pr:23</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>[2025-11-05 pr] “Dynavax Reports Third Quarter 2025 Financial Results and Announces New $100 Million Share Repurchase Program”</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>STGPF ●</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Scentre Group</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>13135.8</v>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:3</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>[2026-04-30 pr] “On April 22, 2026, RE1 Limited, in its capacity as responsible entity and trustee of Scentre Group Trust 2 (the "Offeror"), a trust forming part of the stapled entity Sce”</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>GRNNF ●</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Grand City Properties S.</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>1810.6</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>call:3 pr:1</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-12 call] “In the second quarter, we issued EUR 600 million of new notes at a coupon of 5.25%, following the transaction we executed in the fourth quarter of last year and completed”</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>OILSF ●</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Saturn Oil &amp; Gas Inc.</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>888.1</v>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:19</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>[2026-05-07 call] “Since August of 2025, when we renewed our NCIB, the number of shares we have bought back is nearing the maximum allowable for a 1-year period, equal to 12.1 million share”</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>FMCQF ●</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Fresenius Medical Care A</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>11849.1</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>call:4</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-04 call] “After canceling 8.5% of shares, which we bought back as part of the share buyback program completed in April of this year, we initiated a new share buyback program starti”</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>EOHDF ●</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Emeco Holdings Limited</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>408.6</v>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-19 call] “Given the sustained cash generation and strong balance sheet, the board has approved an on-market share buyback of up to 10% of shares on issue.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>GRWXF ●</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Molten Ventures Ord</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>1550</v>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>[2026-06-09 call] “We still have about GBP 4 million of the most recent announced buyback tranche left to run.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>NPSNY ●</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Naspers Limited</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>6960.6</v>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:1</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>[2026-06-29 call] “On the share buyback — last year we sold about $2 billion from non-core assets, and in the first quarter of this year almost a billion.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>GRGTF ●</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Grainger plc</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>1626.4</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-20 call] “We've done GBP 82 million of sales of our non-core assets and that's either completed or exchanged in the year-to-date.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>NOEJF ●</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>NORMA Group SE</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>538.5</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>call:3</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>[2026-03-31 call] “However, now with the divestment, with the new situation with the new strategy, we will have a good basis for new NORMA, and therefore, we are going to reset and start wi”</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>SPFX ●</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Standard Premium Finance</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>ex99:1 pr:16</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-28 pr] “(OTCQX: SPFX) (“Standard Premium”), a leading specialty finance company, today announces that the Company has repurchased 76,000 shares at $2.25 per share through a board”</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>TWODF ●</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Taylor Wimpey plc</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>3612.5</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>[2026-03-05 call] “Accordingly, today, we are announcing a final 2025 dividend of GBP 0.0295 per share, equivalent to GBP 105 million and a GBP 52 million share buyback, which will commence”</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>KRNGF ●</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Karoon Energy Ltd</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>845.7</v>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-26 call] “Since the 30th of June, we have completed a further USD 15 million buyback tranche, purchasing approximately 12.6 million shares between the 23rd of July and the 7th of A”</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>PAFRY ●</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Pan African Resources PL</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>[2026-09-16 call] “The Board has also approved a share buyback program to purchase up to ZAR 500 million or approximately $30 million of ordinary shares of the company, commencing during Oc”</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>IPXHF ●</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Inpex Corporation</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>30170.4</v>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-07 call] “From that standpoint, we think internally, we think we are undervalued and that is, as a company, the understanding we have today.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ONEXF ●</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Onex Corporation</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>5886.7</v>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:14</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-13 call] “Our strategy will include both share repurchases and deploying capital into 1 or 2 additional investments that can deliver compelling risk-adjusted returns for shareholde”</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>MSADF ●</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>MS&amp;AD Insurance Group Ho</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>46328.5</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-20 call] “In addition to this, we plan to repurchase JPY 80 billion of our own shares during the first half as part of our basic shareholder return and combined with JPY 190 billio”</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>TIHRF ●</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Tharisa plc</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>471.1</v>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>[2026-05-21 call] “Profit before tax, also strongly up at $69.9 million, translating to earnings per share of $0.158 per share, that's up 532% -- and very pleasing, the Board approved an in”</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>LIMAF ●</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Linamar Corporation</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>4057.3</v>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>call:3 pr:11</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>[2025-10-09 pr] “(“Aludyne” or the “Company”), a global lightweighting solutions and components supplier to the mobility industry, today announced that it has entered into a definitive ag”</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>CDEVY ●</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>City Developments Limite</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>5315.7</v>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>call:1</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-12 call] “But anyway, all that we will share more when we release our strategic review outcome end of next month.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>IMPJY ●</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Webuild S.p.A.</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>2305.1</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>call:1</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>[2026-07-30 call] “And in line with the direction of that plan, yesterday, we announced to launch a voluntary tender offer for all the ordinary share of Trevi.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>FRFFF ●</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Fairfax Financial Holdin</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>15669.4</v>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>call:4 pr:6</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-31 call] “So we think it still remains undervalued.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>HDIUF ●</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>ADENTRA Inc.</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>642.3</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-06 call] “During the quarter, we returned approximately $5.6 million to shareholders through dividends and share repurchases.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>PARXF ●</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Parex Resources Inc.</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>1824.5</v>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>call:4 pr:11</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-31 call] “This focus will drive compounding efficiencies and expand our free cash flow profile, giving us the flexibility to reinvest in organic growth, strengthen our balance shee”</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>NHOLF ●</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Sompo Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>39116</v>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-20 call] “As to share buyback, we have decided to buy back shares worth JPY 69 billion for the second half, making the total annual amount JPY 146 billion.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>CKHUF ●</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>CK Hutchison Holdings Li</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G35" s="12" t="n">
+        <v>32517.1</v>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-13 call] “And as a result, they increased their dividend by close to 3% to HKD 0.75, right, marking, I think, the 30th year in a row that we managed to grow and grow dividends in t”</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>VGPBF ●</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Vgp N.V.</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>2488.5</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>call:2 pr:3</t>
+        </is>
+      </c>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-20 call] “And also, we bought back EUR 100 million on the January '27 bond outstanding.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SUMXF ●</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Supremex Inc.</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G37" s="12" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:8</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>[2025-11-06 call] “In this regard, following the launch of a normal course issuer bid program in August, we repurchased approximately 44,000 shares in Q3 for a consideration of $0.2 million”</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>NNGPF ●</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>NN Group N.V.</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>23839</v>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I38" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-06 call] “And we remain firmly committed to extending that track record with total capital return to shareholders foreseen to grow over EUR 15 billion by 2028 based on current comm”</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>ETST ●</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Earth Science Tech, Inc.</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="G39" s="12" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>ex99:9 letter:1 pr:17</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>[2026-06-18 ex99] “During fiscal 2026 and subsequent to year end, we repurchased and retired more than 7.1 million shares of common stock, continued investing in new products and expanded t”</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>CMRB</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>First Commerce Bank</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G40" s="13" t="n">
+        <v>151.9</v>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>pr:10</t>
+        </is>
+      </c>
+      <c r="I40" s="10" t="inlineStr">
+        <is>
+          <t>[2026-03-30 pr] “President &amp; CEO Donald Mindiak commented, "On the heels of a capital raise in the form of a $40.0 million Subordinated Debt Offering, which was noteworthy in that it was ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>AIMFF</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Aimia Inc.</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G41" s="12" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>call:4</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-11 call] “We completed a tender offer to purchase senior notes due in January 2030, reducing our interest costs materially.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>WNDLF</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Wendel</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="G42" s="13" t="n">
+        <v>3549.5</v>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>call:2 pr:17</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
+        <is>
+          <t>[2026-02-26 call] “The sale of Stahl is going to bring $1.2 billion of net proceeds to Wendel and the expected tender offer on IHS should bring $575 million for the shares that we own in IH”</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>LNWO</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Light &amp; Wonder, Inc.</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="G43" s="12" t="n">
+        <v>6215.1</v>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>call:3 ex99:5 pr:7</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-04 call] “Since the inception of our first ever share repurchase program back in 2022, we have returned $2.1 billion to shareholders.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>CURLF</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Curaleaf Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="G44" s="13" t="n">
+        <v>3094.2</v>
+      </c>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t>call:3 pr:66</t>
+        </is>
+      </c>
+      <c r="I44" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-16 pr] “(TSX: CURA) (OTCQX: CURLF ) ("Curaleaf" or the "Company"), a leading international provider of consumer cannabis products, has announced that its Board of Directors has a”</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>CSHX</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Cashmere Valley Bank</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G45" s="12" t="n">
+        <v>333.1</v>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>pr:13</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>[2026-03-18 pr] “Cashmere Valley Bank Commences Self Tender Offer to Repurchase up to 200,000 Shares of its Common Stock”</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>PRPH</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>ProPhase Labs, Inc.</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H46" s="10" t="inlineStr">
+        <is>
+          <t>call:1 pr:14</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="inlineStr">
+        <is>
+          <t>[2025-11-19 call] “Then the Crown Medical, $20 million is going to come in, and I am going to buy back half the shares outstanding in the company.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>LOQPF</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>accesso Technology Group</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G47" s="12" t="n">
+        <v>161.9</v>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:1</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>[2026-03-30 call] “And then on the 18th of March, we completed a tender offer that you will all have seen for $20 million returning or purchasing and canceling 4.8 million shares and just s”</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>BTDPY</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Barratt Redrow PLC Unspo</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>2790.7</v>
+      </c>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
+        <is>
+          <t>[2026-09-16 call] “Over the last 10 years, we have returned nearly GBP 3.5 billion to shareholders, with GBP 1 billion returned through share buyback or special dividends.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>CLILF</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>CapitaLand Investment Li</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G49" s="12" t="n">
+        <v>10225.1</v>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-12 call] “Private funds contribution has increased, is expected to also increase going forward as we've been divesting some of our lower-yielding assets and reinvesting into credit”</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>VREOF</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>Vireo Growth Inc.</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>453.7</v>
+      </c>
+      <c r="H50" s="10" t="inlineStr">
+        <is>
+          <t>call:2 ex99:10 pr:32</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-18 ex99] “("Vireo" or the "Company") (CSE: VREO; OTCQX: VREOF), a leading vertically integrated cannabis company and agricultural markets platform, today announced it has received ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>EXXRF</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Exor N.V.</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G51" s="12" t="n">
+        <v>16714.5</v>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:9</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>[2026-09-23 call] “You'll see also in the announcement that we are very explicit that both because the shares trade at a substantial discount to our NAV and don't reflect our assessment of ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>SGBAF</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Ses S.a.</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>2311.8</v>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>call:4 pr:100</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>[2026-07-31 pr] “In the time period from June 2, 2026 until and including June 23, 2026, a number of 213,167 shares were bought back within the framework of the share buyback of SES to me”</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>EUZOF</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Eurazeo SE</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G53" s="12" t="n">
+        <v>2936.7</v>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-23 call] “In 2026, we have already distributed a dividend per share increasing by 10% and executed half of the share buyback program for the year.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>MUEL</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Paul Mueller Company</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="G54" s="13" t="n">
+        <v>594.3</v>
+      </c>
+      <c r="H54" s="10" t="inlineStr">
+        <is>
+          <t>pr:13</t>
+        </is>
+      </c>
+      <c r="I54" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-07 pr] “Paul Mueller Company (OTC: MUEL) (the “Company”) today announced that the Board of Directors has approved a tender offer (the “Tender Offer”) to repurchase up to 35,000 s”</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>UTGPF</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Unite Group Plc</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G55" s="12" t="n">
+        <v>3437.4</v>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>call:2 pr:23</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-28 call] “We've completed GBP 165 million of share buybacks in H1, and we still see Unite shares as the best way for us to invest in high-quality student accommodation today.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>LTUM</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Lithium Corporation</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="F56" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G56" s="13" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H56" s="10" t="inlineStr">
+        <is>
+          <t>pr:100</t>
+        </is>
+      </c>
+      <c r="I56" s="10" t="inlineStr">
+        <is>
+          <t>[2026-09-10 pr] “To exercise the Option and acquire a 100% interest in the Property, Osisko must: (a) make the following cash payments to the Company: (i) $100,000 on the Effective Date; ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>APNHY</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Aspen Pharmacare Holding</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G57" s="12" t="n">
+        <v>4462.4</v>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>[2026-09-03 call] “And as we said, we -- I think as at 2 days ago, we announced a 3% share buyback at ZAR 2 billion of investment.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>RHEPB</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Regional Health Properti</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="G58" s="13" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>ex99:3</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>[2025-12-01 ex99] “(the “Company”, “Regional”, “we”, “us” or “our”) (OTCQB: RHEP) (OTCQB: RHEPA) (OTCQB: RHEPB) (OTCQB:RHEPZ), today announced that its Board of Directors authorized and app”</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>BTRCF</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Better Collective A/S</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G59" s="12" t="n">
+        <v>881.1</v>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>call:4</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>[2026-05-21 call] “In March, we launched a new share buyback program of up to EUR 40 million.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>GTBIF</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Green Thumb Industries I</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G60" s="13" t="n">
+        <v>1677.5</v>
+      </c>
+      <c r="H60" s="10" t="inlineStr">
+        <is>
+          <t>call:1 ex99:5 pr:17</t>
+        </is>
+      </c>
+      <c r="I60" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-06 ex99] “• Repurchased approximately 7.4 million additional Subordinate Voting Shares, bringing 2026 year-to-date repurchases to approximately 13.4 million Subordinate Voting Shar”</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>ZSPC</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>zSpace, Inc.</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>call:3 ex99:7 pr:100</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>[2026-05-14 ex99] “Board of Directors Launches Strategic Alternatives Review to Unlock Shareholder Value”</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>FBBPF</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>FIBRA Prologis</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E62" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G62" s="13" t="n">
+        <v>7256.7</v>
+      </c>
+      <c r="H62" s="10" t="inlineStr">
+        <is>
+          <t>call:4 pr:23</t>
+        </is>
+      </c>
+      <c r="I62" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-30 call] “We will eventually sell our non-core portfolio.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>OTCM</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>OTC Markets Group Inc.</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="G63" s="12" t="n">
+        <v>662.2</v>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:87</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>[2026-03-05 call] “During 2025, we returned a total of $32,600,000 to investors in the form of dividends and through our stock buyback program, a 10% increase from the prior year primarily ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>VTMTF</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Vertu Motors plc</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G64" s="13" t="n">
+        <v>360</v>
+      </c>
+      <c r="H64" s="10" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I64" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-18 call] “And to date, we have in the form of dividends and buybacks, returned GBP 112 million in cash, reflecting the strong underlying cash flows of the group.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>ALYAF</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Alithya Group Inc.</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G65" s="12" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:12</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>[2026-02-13 call] “In connection with the Datum transaction that Paul alluded to earlier, we will be repurchasing close to 2.5 million Class A shares from Amar.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>CCFN</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>Muncy Columbia Financial</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="G66" s="13" t="n">
+        <v>323.7</v>
+      </c>
+      <c r="H66" s="10" t="inlineStr">
+        <is>
+          <t>ex99:8 letter:1 pr:9</t>
+        </is>
+      </c>
+      <c r="I66" s="10" t="inlineStr">
+        <is>
+          <t>[2026-05-12 ex99] “The program authorizes the repurchase of up to an additional 530,611 shares, or 5% of the Corporation's issued and outstanding common shares as of May 15, 2026.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>VSTKF</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>VNV Global AB (publ)</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G67" s="12" t="n">
+        <v>252.2</v>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>call:4</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>[2026-04-22 call] “Also sort of during the quarter, we bought back another close to 500,000 VNV shares and also a small amount of the outstanding bonds, which I'll come to now, which we als”</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>BKSC</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Bank of South Carolina C</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G68" s="13" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="H68" s="10" t="inlineStr">
+        <is>
+          <t>pr:9</t>
+        </is>
+      </c>
+      <c r="I68" s="10" t="inlineStr">
+        <is>
+          <t>[2025-12-18 pr] “This new repurchase program replaces the previous stock repurchase program approved by the Board on May 25, 2023, which recently concluded with the successful repurchase ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>DEXSF</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Dexus</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G69" s="12" t="n">
+        <v>4105.3</v>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-20 call] “So, I think we see opportunity to sell assets where kind of the go-forward returns are going to not meet our hurdles or returns relative to the redeployment opportunities”</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>ENTOF</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Entra ASA</t>
+        </is>
+      </c>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G70" s="13" t="n">
+        <v>2034.8</v>
+      </c>
+      <c r="H70" s="10" t="inlineStr">
+        <is>
+          <t>call:3</t>
+        </is>
+      </c>
+      <c r="I70" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-21 call] “Divestments of negative NOK 553 million is related to the Christian Krohgs gate 2 project or joint venture project we have with Skanska, which we announced in the fourth ”</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>GLXZ</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Galaxy Gaming, Inc.</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G71" s="12" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>ex99:6 pr:9</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-22 ex99] “GALAXY GAMING BOARD AUTHORIZES $4 MILLION SHARE REPURCHASE PROGRAM”</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>PRTCY</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>PureTech Health plc</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E72" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F72" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G72" s="13" t="n">
+        <v>375.2</v>
+      </c>
+      <c r="H72" s="10" t="inlineStr">
+        <is>
+          <t>call:2 pr:1</t>
+        </is>
+      </c>
+      <c r="I72" s="10" t="inlineStr">
+        <is>
+          <t>[2026-09-22 call] “In practice, this means that we will prioritize maintaining an appropriate operational runway, selectively deploying capital where we see compelling risk-adjusted opportu”</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>SMBMF</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Seatrium Limited</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G73" s="12" t="n">
+        <v>5286.4</v>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-30 call] “Upon completion, we intend to launch a new share buyback program to enhance shareholder value.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>ONEI</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>OneMeta AI</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="F74" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G74" s="13" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H74" s="10" t="inlineStr">
+        <is>
+          <t>ex99:1 pr:13</t>
+        </is>
+      </c>
+      <c r="I74" s="10" t="inlineStr">
+        <is>
+          <t>[2026-04-14 pr] “The Company repurchased 4,166,667 shares of its Series B-1 Preferred Stock for an aggregate purchase price of $2,750,000.22.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>CCGPY</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>C&amp;C Group plc</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G75" s="12" t="n">
+        <v>540.4</v>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>[2025-10-27 call] “Clearly, our preference is for the former, and we completed the latest EUR 15 million tranche of share buybacks in September of this year.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>RIOCF</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>RioCan Real Estate Inves</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E76" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G76" s="13" t="n">
+        <v>4275</v>
+      </c>
+      <c r="H76" s="10" t="inlineStr">
+        <is>
+          <t>call:3 pr:28</t>
+        </is>
+      </c>
+      <c r="I76" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-04 call] “This extends beyond operations to capital allocation, where we've made significant progress, including the near completion of the RioCan Living portfolio monetization.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>MBAK</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>MBAK Energy Solutions In</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>pr:9</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>[2026-02-03 pr] “(OTC:MBAK) Announces $500,000 Share Repurchase Plan”</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>AAWH</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Ascend Wellness Holdings</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F78" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G78" s="13" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="H78" s="10" t="inlineStr">
+        <is>
+          <t>call:3 ex99:1 pr:18</t>
+        </is>
+      </c>
+      <c r="I78" s="10" t="inlineStr">
+        <is>
+          <t>[2025-11-10 call] “Since the launch of the buyback initiative last year, we have repurchased and retired approximately 5 million shares at an average price of $0.30 per share.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>LLESF</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Lendlease Group</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G79" s="12" t="n">
+        <v>1354.1</v>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>call:2</t>
+        </is>
+      </c>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>[2026-08-19 call] “We're looking to take costs out of that ahead of asset sales, and then that will wind down with asset sales.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>HUSQF</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Husqvarna AB</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E80" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G80" s="13" t="n">
+        <v>2356.1</v>
+      </c>
+      <c r="H80" s="10" t="inlineStr">
+        <is>
+          <t>call:4 pr:1</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>[2026-07-17 call] “Today, we also announced that we will move from a turnaround case to a strategic review of our Powered Garden business portfolio unit within the Gardena division.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>CIBH</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>CIB Marine Bancshares, I</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G81" s="12" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>pr:7</t>
+        </is>
+      </c>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>[2026-05-01 pr] “As a result, the total amount authorized for the repurchase of the Company's outstanding common stock has increased from $2.5 million to $3.5 million with the program con”</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>CVAT</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>Cavitation Technologies,</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E82" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G82" s="13" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="H82" s="10" t="inlineStr">
+        <is>
+          <t>ex99:1 pr:13</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>[2026-08-19 ex99] “(OTCQB: CVAT) ("CVAT" or the "Company"), a leading provider of sustainable nanotechnology solutions, today announced that, on August 14, 2026, the Company executed a defi”</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>SCBFF</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Standard Chartered PLC</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G83" s="12" t="n">
+        <v>65112.2</v>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>call:3 pr:9</t>
+        </is>
+      </c>
+      <c r="I83" s="7" t="inlineStr">
+        <is>
+          <t>[2026-07-29 call] “And even after today, we'll still be very happy to buy back $1 billion of shares at this price.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>AAVVF</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>Advantage Energy Ltd.</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>ACT SIGNALLED</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G84" s="13" t="n">
+        <v>1197.9</v>
+      </c>
+      <c r="H84" s="10" t="inlineStr">
+        <is>
+          <t>call:3</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr">
+        <is>
+          <t>[2026-07-31 call] “Share buybacks are going to be our main vehicle for shareholder returns while our shares are trading below intrinsic value.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>244 OTC names with a current intent signal (ACT SIGNALLED = top decile with a realised/committed shareholder action, a NEW family vs the prior 12 months, or a stated buyback/tender &gt;= 5% of mcap; BUILDING = top quartile; last document &lt;= 200 days old). Weights come from the earnings-call validation (tender 2.2x, buyback/dividend 1.6x, value-gap 1.4x lift for subsequent action). Language predicts ACTION, not the re-rating by itself — pair it with the cheapness tabs. See OTC_INTENT_VALIDATION.md. Source: otc_comms.py.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A86:I86"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>